<commit_message>
Revert "fix(qa): marcar bugs P1 backoffice como solucionados con descripcion del fix"
This reverts commit d24a39f3b4685fbf4bbbe466c1718631a0348a0c.
</commit_message>
<xml_diff>
--- a/Web/TestCasesWeb/Login.xlsx
+++ b/Web/TestCasesWeb/Login.xlsx
@@ -1,72 +1,172 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nerea QA\PycharmProjects\KOVAI\Web\TestCases\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16124479-D56A-43C6-A652-B6BB9822B013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1950" yWindow="1950" windowWidth="26850" windowHeight="8040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="26850" windowHeight="8040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="31">
+  <si>
+    <t>Num</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Summary</t>
+  </si>
+  <si>
+    <t>Pasos</t>
+  </si>
+  <si>
+    <t>I try to login with wrong user</t>
+  </si>
+  <si>
+    <t>I try to login with wrong password</t>
+  </si>
+  <si>
+    <t>I do login</t>
+  </si>
+  <si>
+    <t>Expected Result</t>
+  </si>
+  <si>
+    <t>Obtained Result</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>1. The user logs in successfully.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. The user sees the Login page
+2. The user introduces user and pwd </t>
+  </si>
+  <si>
+    <t>1. The user sees the Login page
+2.  The user to login with wrong user</t>
+  </si>
+  <si>
+    <t>1. The user sees the Login page
+2.  The user to login with wrong password</t>
+  </si>
+  <si>
+    <t>1. The user sees the Login page
+2. The user to login without password</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>KO</t>
+  </si>
+  <si>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>The message shown is: [object Object]</t>
+  </si>
+  <si>
+    <t>The user can not do log in.
+An error is not shown</t>
+  </si>
+  <si>
+    <t>1. The user can not do log in.
+2. An error is shown.</t>
+  </si>
+  <si>
+    <t>I try to login without user/password</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Cxs_yuyLHFT1JsmgWJW-SEwL_8VR9ryI/view?usp=drive_link</t>
+  </si>
+  <si>
+    <t>LOGIN001</t>
+  </si>
+  <si>
+    <t>LOGIN002</t>
+  </si>
+  <si>
+    <t>LOGIN003</t>
+  </si>
+  <si>
+    <t>LOGIN004</t>
+  </si>
+  <si>
+    <t>Login page home</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. The user sees the Login page
+</t>
+  </si>
+  <si>
+    <t>1. The login page home is correctly.</t>
+  </si>
+  <si>
+    <t>LOGIN005</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="6">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
     <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
     <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="10"/>
-      <sz val="11"/>
-      <u val="single"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <sz val="8"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00276221"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -95,30 +195,27 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -140,7 +237,19 @@
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF6565"/>
+    </mruColors>
+  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -428,258 +537,171 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col width="14.42578125" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="41.5703125" customWidth="1" min="4" max="4"/>
-    <col width="33.42578125" customWidth="1" min="5" max="6"/>
-    <col width="91.42578125" bestFit="1" customWidth="1" min="8" max="8"/>
+    <col min="2" max="2" width="14.42578125" customWidth="1"/>
+    <col min="3" max="3" width="48" customWidth="1"/>
+    <col min="4" max="4" width="41.5703125" customWidth="1"/>
+    <col min="5" max="6" width="33.42578125" customWidth="1"/>
+    <col min="8" max="8" width="91.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Num</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Pasos</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Expected Result</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Obtained Result</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="H1" s="4" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="2" t="n">
+    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN001</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Login page home</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. The user sees the Login page
-</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>1. The login page home is correctly.</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H2" s="1" t="n"/>
+      <c r="B2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="3"/>
+      <c r="G2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" s="1"/>
     </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="2" t="n">
+    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN002</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>I do login</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1. The user sees the Login page
-2. The user introduces user and pwd </t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>1. The user logs in successfully.</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H3" s="1" t="n"/>
+      <c r="B3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="1"/>
     </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="2" t="n">
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN003</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>I try to login with wrong user</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>1. The user sees the Login page
-2.  The user to login with wrong user</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>1. The user can not do log in.
-2. An error is shown.</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Se muestra correctamente el mensaje de error del servidor</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>SOLUCIONADO: El interceptor de Axios en api.ts ya no intercepta las llamadas a /auth/login para intentar refresh, por lo que el error 401 llega al store y se muestra correctamente en el formulario de login.</t>
-        </is>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>22</v>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="2" t="n">
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN004</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>I try to login with wrong password</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>1. The user sees the Login page
-2.  The user to login with wrong password</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>1. The user can not do log in.
-2. An error is shown.</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Se muestra el mensaje de error al fallar la autenticación</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>FIXED</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>SOLUCIONADO: Mismo fix que LOGIN003. La función getErrorMessage en auth.store.ts también se hizo más defensiva para manejar cualquier formato de mensaje del backend.</t>
-        </is>
-      </c>
+      <c r="B5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="2"/>
     </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="2" t="n">
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>LOGIN005</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>I try to login without user/password</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>1. The user sees the Login page
-2. The user to login without password</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>1. The user can not do log in.
-2. An error is shown.</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="4" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n"/>
+      <c r="B6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F6" s="3"/>
+      <c r="G6" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="H6" s="2"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="G2:G6">
-    <cfRule type="containsText" priority="1" operator="containsText" dxfId="1" text="KO">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="KO">
       <formula>NOT(ISERROR(SEARCH("KO",G2)))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="3" operator="containsText" dxfId="0" text="OK">
+    <cfRule type="containsText" dxfId="0" priority="3" operator="containsText" text="OK">
       <formula>NOT(ISERROR(SEARCH("OK",G2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId1"/>
+    <hyperlink ref="H4" r:id="rId1" xr:uid="{7414C937-D2D7-4D9C-BADD-CF4D3CE8EE08}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>